<commit_message>
chore: add database migration for mandor task notes and photos and update operator data
</commit_message>
<xml_diff>
--- a/prisma/csv/data_operator.xlsx
+++ b/prisma/csv/data_operator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\0Magang\Toshin-Backend\prisma\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEF99D36-4F25-4F80-9DF5-067CE76C08B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F89C595-5C72-468C-BB16-310809B52E8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{09414138-216C-42B7-9765-4E788DA6B58B}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="25600" windowHeight="14350" xr2:uid="{09414138-216C-42B7-9765-4E788DA6B58B}"/>
   </bookViews>
   <sheets>
     <sheet name="Operator" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1231" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1231" uniqueCount="399">
   <si>
     <t>Line</t>
   </si>
@@ -1229,6 +1229,9 @@
   </si>
   <si>
     <t>1106007</t>
+  </si>
+  <si>
+    <t>MANDOR</t>
   </si>
 </sst>
 </file>
@@ -1798,7 +1801,7 @@
         <v>123</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>262</v>
+        <v>398</v>
       </c>
       <c r="D4" s="2">
         <v>3</v>
@@ -1809,9 +1812,9 @@
       <c r="F4" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="G4" s="16">
+      <c r="G4" s="16" t="e">
         <f>_xlfn.XLOOKUP(C4,'Master Divisi'!B:B,'Master Divisi'!A:A)</f>
-        <v>1</v>
+        <v>#N/A</v>
       </c>
       <c r="H4" s="20">
         <v>17040094</v>

</xml_diff>